<commit_message>
implement V_cap and M_cap structural capacity checks for FEM piles
Add per-element shear and moment capacity checks in the viscoplastic
iteration loop. When lateral force exceeds V_cap/S or moment exceeds
M_cap/S, corrections are applied as equivalent nodal loads (same
pattern as reinforcement). Forces are capped at capacity (elastic-
perfectly-plastic behavior). Summary reports capacity limits, yielded
element counts, and per-element status.

Also fix mesh.py: snap constraint line endpoints to nearby polygon
boundary points to prevent near-zero-length elements when pile top
coordinates don't exactly match the ground surface. Add zero-length
element filtering for both linear and quadratic 1D elements.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fem/files/xslope_piles_fem.xlsx
+++ b/docs/fem/files/xslope_piles_fem.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/fem/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/lem/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB89E2EC-4267-B542-9954-775340309466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC80A1D-6F0F-7946-B56C-42AA61D9EA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31100" yWindow="5880" windowWidth="37700" windowHeight="20620" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="14000" yWindow="2020" windowWidth="42700" windowHeight="22800" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="182">
   <si>
     <t>X</t>
   </si>
@@ -696,15 +696,9 @@
     <t>Polygon #15</t>
   </si>
   <si>
-    <t>label</t>
-  </si>
-  <si>
     <t>H</t>
   </si>
   <si>
-    <t>theta</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
@@ -714,13 +708,47 @@
     <t>I</t>
   </si>
   <si>
-    <t>Required for LEM only</t>
-  </si>
-  <si>
-    <t>Optional</t>
-  </si>
-  <si>
     <t xml:space="preserve">Polygons coordinates can be input in CW or CCW order. </t>
+  </si>
+  <si>
+    <t>Vcap</t>
+  </si>
+  <si>
+    <t>Mcap</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>q</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>p</t>
+    </r>
+  </si>
+  <si>
+    <t>LEM only</t>
+  </si>
+  <si>
+    <t>LEM &amp; FEM</t>
+  </si>
+  <si>
+    <t>FEM only</t>
   </si>
   <si>
     <t>soil</t>
@@ -733,7 +761,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -856,6 +884,13 @@
       <sz val="12"/>
       <color theme="0"/>
       <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Symbol"/>
+      <charset val="2"/>
     </font>
   </fonts>
   <fills count="17">
@@ -1042,7 +1077,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1164,11 +1199,16 @@
     <xf numFmtId="0" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1177,10 +1217,7 @@
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1207,11 +1244,68 @@
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="17">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -8290,7 +8384,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000039-E198-1942-8CC0-5F5B615D56D7}"/>
+                <c16:uniqueId val="{00000039-9273-8E45-8E0C-DF8E6C08CDD2}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -8438,673 +8532,6 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000050-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="87"/>
-          <c:order val="87"/>
-          <c:tx>
-            <c:v>Pile #11</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent4">
-                    <a:lumMod val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:dPt>
-            <c:idx val="0"/>
-            <c:marker>
-              <c:symbol val="circle"/>
-              <c:size val="5"/>
-              <c:spPr>
-                <a:solidFill>
-                  <a:schemeClr val="accent4">
-                    <a:lumMod val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:ln w="9525">
-                  <a:solidFill>
-                    <a:schemeClr val="accent4">
-                      <a:lumMod val="50000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-            </c:marker>
-            <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent4">
-                    <a:lumMod val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:round/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:extLst>
-              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000003B-E198-1942-8CC0-5F5B615D56D7}"/>
-              </c:ext>
-            </c:extLst>
-          </c:dPt>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$13,piles!$E$13)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$13,piles!$F$13)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000051-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="88"/>
-          <c:order val="88"/>
-          <c:tx>
-            <c:v>Pile #12</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:lumMod val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$14,piles!$E$14)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$14,piles!$F$14)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000052-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="89"/>
-          <c:order val="89"/>
-          <c:tx>
-            <c:v>Pile #13</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent6">
-                    <a:lumMod val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$15,piles!$E$15)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$15,piles!$F$15)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000053-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="90"/>
-          <c:order val="90"/>
-          <c:tx>
-            <c:v>Pile #14</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$16,piles!$E$16)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$16,piles!$F$16)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000054-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="91"/>
-          <c:order val="91"/>
-          <c:tx>
-            <c:v>Pile #15</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent2">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$17,piles!$E$17)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$17,piles!$F$17)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000055-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="92"/>
-          <c:order val="92"/>
-          <c:tx>
-            <c:v>Pile #16</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent3">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent3">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$18,piles!$E$18)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$18,piles!$F$18)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000056-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="93"/>
-          <c:order val="93"/>
-          <c:tx>
-            <c:v>Pile #17</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent4">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$19,piles!$E$19)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$19,piles!$F$19)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000057-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="94"/>
-          <c:order val="94"/>
-          <c:tx>
-            <c:v>Pile #18</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$20,piles!$E$20)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$20,piles!$F$20)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000058-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="95"/>
-          <c:order val="95"/>
-          <c:tx>
-            <c:v>Pile #19</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="70000"/>
-                  <a:lumOff val="30000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent6">
-                    <a:lumMod val="70000"/>
-                    <a:lumOff val="30000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$21,piles!$E$21)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$21,piles!$F$21)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000059-A2F6-274C-9E15-3D60CC318540}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="96"/>
-          <c:order val="96"/>
-          <c:tx>
-            <c:v>Pile #20</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="70000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="70000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="70000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>(piles!$C$22,piles!$E$22)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>(piles!$D$22,piles!$F$22)</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000005A-A2F6-274C-9E15-3D60CC318540}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -9932,13 +9359,13 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>553357</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>99787</xdr:rowOff>
+      <xdr:rowOff>99788</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>780143</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>54428</xdr:rowOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>181429</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -9953,8 +9380,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9180286" y="498930"/>
-          <a:ext cx="4354286" cy="2748641"/>
+          <a:off x="9180286" y="498931"/>
+          <a:ext cx="4354286" cy="1877784"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10002,20 +9429,14 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
-        </a:p>
-        <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>Tmax</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> = maximum tensile strength of reinforcement material. </a:t>
+            <a:t> = maximum tensile strength (per unit width) of reinforcement material. </a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -10024,11 +9445,8 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> = residual strenth of reinfocement material.</a:t>
+            <a:t> = residual strenth (per unit width) of reinfocement material.</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -10043,9 +9461,6 @@
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
             <a:t> length or length required to generate full frictional resistance on end corresponding to point 1.</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
@@ -10079,20 +9494,31 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
-        </a:p>
-        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>E</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> = modulus of elasticity of reinforcement material</a:t>
+            <a:t> = Young's modulus of reinforcement material (force/length^2)</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -10101,7 +9527,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> = cross-sectional area (per unit width) of reinforcement material </a:t>
+            <a:t> = cross-sectional area (per unit width) of reinforcement material.</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
@@ -10116,16 +9542,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>553357</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>99787</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>290285</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>18144</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>27214</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>54428</xdr:rowOff>
+      <xdr:colOff>680357</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -10140,8 +9566,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10885714" y="498930"/>
-          <a:ext cx="4426857" cy="2748641"/>
+          <a:off x="12273642" y="217715"/>
+          <a:ext cx="3156858" cy="1841499"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10189,9 +9615,6 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
-        </a:p>
-        <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>H</a:t>
@@ -10202,12 +9625,15 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
-        </a:p>
-        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:latin typeface="Symbol" pitchFamily="2" charset="2"/>
+            </a:rPr>
+            <a:t>q</a:t>
+          </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t>theta</a:t>
+            <a:t>p</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
@@ -10223,11 +9649,8 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Force angle from horizontal in degrees (default 0°; positive = upward)</a:t>
+            <a:t>Force angle from horizontal in degrees (degrees)</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -10248,11 +9671,29 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Pile diameter.</a:t>
+            <a:t>Pile diameter</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> (ft or m)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
@@ -10282,11 +9723,8 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>.</a:t>
+            <a:t> (ft or m)</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -10295,11 +9733,8 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> = Young's modulus of pile material</a:t>
+            <a:t> = Young's modulus of pile material (force/lengh^2)</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
         </a:p>
         <a:p>
           <a:r>
@@ -10320,43 +9755,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Moment of inertia (computed from</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> D</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="ar-AE" sz="1100" b="0" i="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>if omitted)</a:t>
+            <a:t>Moment of inertia (length^4)</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
             <a:solidFill>
@@ -10369,9 +9768,6 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
-        </a:p>
-        <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>Area</a:t>
@@ -10390,10 +9786,12 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Cross-sectional area (computed from</a:t>
+            <a:t>Cross-sectional area (length^2)</a:t>
           </a:r>
+        </a:p>
+        <a:p>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+            <a:rPr lang="en-US" sz="1100" b="1" i="0">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -10402,10 +9800,10 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> D</a:t>
+            <a:t>Vcap</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="ar-AE" sz="1100" b="0" i="0">
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -10414,10 +9812,10 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> </a:t>
+            <a:t> = Shear</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -10426,7 +9824,33 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>if omitted)</a:t>
+            <a:t> capacity of pile (force)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Mcap</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> = Moment capacity of pile (force x length)</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
@@ -10783,11 +10207,11 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="50"/>
-      <c r="D7" s="50"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -11433,9 +10857,10 @@
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="11" width="10.83203125" style="1"/>
+    <col min="12" max="12" width="7.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
@@ -11470,7 +10895,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -11485,7 +10910,7 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -11500,7 +10925,7 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -11515,7 +10940,7 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -11530,7 +10955,7 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -11545,7 +10970,7 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -11560,7 +10985,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -11575,7 +11000,7 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -11590,7 +11015,7 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -11605,7 +11030,7 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -11620,7 +11045,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -11635,7 +11060,7 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -11649,8 +11074,12 @@
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M14" s="31"/>
+      <c r="N14" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -11664,8 +11093,12 @@
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M15" s="34"/>
+      <c r="N15" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -11680,7 +11113,7 @@
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -11695,7 +11128,7 @@
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -11710,7 +11143,7 @@
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -11724,12 +11157,8 @@
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
-      <c r="M19" s="31"/>
-      <c r="N19" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -11743,12 +11172,8 @@
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
-      <c r="M20" s="34"/>
-      <c r="N20" s="9" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -11763,7 +11188,7 @@
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -11778,11 +11203,11 @@
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
     </row>
@@ -11794,20 +11219,21 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C542BD7-5686-4248-AC02-D49DB39A8FC0}">
-  <dimension ref="A2:P25"/>
+  <dimension ref="A2:R15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.5" style="1" customWidth="1"/>
-    <col min="3" max="13" width="10.83203125" style="1"/>
+    <col min="3" max="15" width="10.83203125" style="1"/>
+    <col min="16" max="16" width="3.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C2" s="12" t="s">
         <v>103</v>
@@ -11822,33 +11248,39 @@
         <v>106</v>
       </c>
       <c r="G2" s="45" t="s">
+        <v>168</v>
+      </c>
+      <c r="H2" s="45" t="s">
+        <v>176</v>
+      </c>
+      <c r="I2" s="32" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="32" t="s">
+      <c r="J2" s="32" t="s">
         <v>170</v>
-      </c>
-      <c r="I2" s="32" t="s">
-        <v>171</v>
-      </c>
-      <c r="J2" s="32" t="s">
-        <v>172</v>
       </c>
       <c r="K2" s="33" t="s">
         <v>101</v>
       </c>
       <c r="L2" s="33" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="M2" s="33" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N2" s="46" t="s">
+        <v>173</v>
+      </c>
+      <c r="O2" s="46" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C3" s="3">
         <v>10</v>
@@ -11875,8 +11307,14 @@
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N3" s="3">
+        <v>25000</v>
+      </c>
+      <c r="O3" s="3">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -11892,8 +11330,10 @@
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -11909,8 +11349,10 @@
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -11926,8 +11368,10 @@
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -11943,8 +11387,10 @@
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -11960,8 +11406,10 @@
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -11977,8 +11425,10 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -11994,8 +11444,10 @@
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -12011,8 +11463,10 @@
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -12028,196 +11482,30 @@
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
-        <v>11</v>
-      </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
-        <v>12</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
-        <v>13</v>
-      </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="3">
-        <v>14</v>
-      </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A17" s="3">
-        <v>15</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A18" s="3">
-        <v>16</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A19" s="3">
-        <v>17</v>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="O19" s="46"/>
-      <c r="P19" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A20" s="3">
-        <v>18</v>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
-      <c r="O20" s="31"/>
-      <c r="P20" s="9" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A21" s="3">
-        <v>19</v>
-      </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
-      <c r="O21" s="34"/>
-      <c r="P21" s="9" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A22" s="3">
-        <v>20</v>
-      </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="Q12" s="60"/>
+      <c r="R12" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Q13" s="31"/>
+      <c r="R13" s="9" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="Q14" s="34"/>
+      <c r="R14" s="9" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13098,36 +12386,36 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="C7" s="51" t="s">
+      <c r="C7" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
-      <c r="G7" s="51"/>
-      <c r="H7" s="51"/>
-      <c r="I7" s="51"/>
-      <c r="J7" s="51"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="51" t="s">
+      <c r="L7" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="51"/>
-      <c r="N7" s="51"/>
-      <c r="O7" s="51"/>
-      <c r="P7" s="51"/>
-      <c r="Q7" s="51"/>
-      <c r="R7" s="51" t="s">
+      <c r="M7" s="48"/>
+      <c r="N7" s="48"/>
+      <c r="O7" s="48"/>
+      <c r="P7" s="48"/>
+      <c r="Q7" s="48"/>
+      <c r="R7" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="S7" s="51"/>
-      <c r="T7" s="51"/>
-      <c r="U7" s="51"/>
-      <c r="V7" s="51"/>
-      <c r="W7" s="51" t="s">
+      <c r="S7" s="48"/>
+      <c r="T7" s="48"/>
+      <c r="U7" s="48"/>
+      <c r="V7" s="48"/>
+      <c r="W7" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="X7" s="51"/>
+      <c r="X7" s="48"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
@@ -13208,7 +12496,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C9" s="3">
         <v>120</v>
@@ -13919,33 +13207,38 @@
     <mergeCell ref="W7:X7"/>
     <mergeCell ref="R7:V7"/>
   </mergeCells>
-  <conditionalFormatting sqref="F9:F50">
-    <cfRule type="expression" dxfId="8" priority="1">
-      <formula>$D9="cp"</formula>
+  <conditionalFormatting sqref="F10:F50">
+    <cfRule type="expression" dxfId="16" priority="4">
+      <formula>$D10="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9:H50">
-    <cfRule type="expression" dxfId="7" priority="3">
+    <cfRule type="expression" dxfId="15" priority="3">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:J50">
-    <cfRule type="expression" dxfId="6" priority="5">
+    <cfRule type="expression" dxfId="14" priority="5">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N9:N50">
-    <cfRule type="expression" dxfId="5" priority="7">
+    <cfRule type="expression" dxfId="13" priority="7">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9:O50">
-    <cfRule type="expression" dxfId="4" priority="14">
+    <cfRule type="expression" dxfId="12" priority="14">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P9:Q50">
-    <cfRule type="expression" dxfId="3" priority="9">
+    <cfRule type="expression" dxfId="11" priority="9">
+      <formula>$D9="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F9">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13999,74 +13292,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="D4" s="47" t="s">
+      <c r="B4" s="51"/>
+      <c r="D4" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="47"/>
-      <c r="G4" s="47" t="s">
+      <c r="E4" s="51"/>
+      <c r="G4" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="47"/>
-      <c r="J4" s="47" t="s">
+      <c r="H4" s="51"/>
+      <c r="J4" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="47"/>
-      <c r="M4" s="47" t="s">
+      <c r="K4" s="51"/>
+      <c r="M4" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="47"/>
-      <c r="P4" s="47" t="s">
+      <c r="N4" s="51"/>
+      <c r="P4" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="47"/>
+      <c r="Q4" s="51"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="47" t="s">
+      <c r="S4" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="47"/>
+      <c r="T4" s="51"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="47" t="s">
+      <c r="V4" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="47"/>
+      <c r="W4" s="51"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="47" t="s">
+      <c r="Y4" s="51" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="47"/>
+      <c r="Z4" s="51"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="47" t="s">
+      <c r="AB4" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="47"/>
-      <c r="AE4" s="47" t="s">
+      <c r="AC4" s="51"/>
+      <c r="AE4" s="51" t="s">
         <v>114</v>
       </c>
-      <c r="AF4" s="47"/>
+      <c r="AF4" s="51"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="47" t="s">
+      <c r="AH4" s="51" t="s">
         <v>115</v>
       </c>
-      <c r="AI4" s="47"/>
+      <c r="AI4" s="51"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="47" t="s">
+      <c r="AK4" s="51" t="s">
         <v>116</v>
       </c>
-      <c r="AL4" s="47"/>
+      <c r="AL4" s="51"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="47" t="s">
+      <c r="AN4" s="51" t="s">
         <v>117</v>
       </c>
-      <c r="AO4" s="47"/>
+      <c r="AO4" s="51"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="47" t="s">
+      <c r="AQ4" s="51" t="s">
         <v>118</v>
       </c>
-      <c r="AR4" s="47"/>
+      <c r="AR4" s="51"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -14169,89 +13462,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="48" t="str">
+      <c r="A6" s="49" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>soil</v>
       </c>
-      <c r="B6" s="49"/>
-      <c r="D6" s="48" t="str">
+      <c r="B6" s="50"/>
+      <c r="D6" s="49" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="49"/>
-      <c r="G6" s="48" t="str">
+      <c r="E6" s="50"/>
+      <c r="G6" s="49" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="49"/>
-      <c r="J6" s="48" t="str">
+      <c r="H6" s="50"/>
+      <c r="J6" s="49" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="49"/>
-      <c r="M6" s="48" t="str">
+      <c r="K6" s="50"/>
+      <c r="M6" s="49" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="49"/>
-      <c r="P6" s="48" t="str">
+      <c r="N6" s="50"/>
+      <c r="P6" s="49" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="49"/>
+      <c r="Q6" s="50"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="48" t="str">
+      <c r="S6" s="49" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="49"/>
+      <c r="T6" s="50"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="48" t="str">
+      <c r="V6" s="49" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="49"/>
+      <c r="W6" s="50"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="48" t="str">
+      <c r="Y6" s="49" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="49"/>
+      <c r="Z6" s="50"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="48" t="str">
+      <c r="AB6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="49"/>
-      <c r="AE6" s="48" t="str">
+      <c r="AC6" s="50"/>
+      <c r="AE6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="49"/>
+      <c r="AF6" s="50"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="48" t="str">
+      <c r="AH6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="49"/>
+      <c r="AI6" s="50"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="48" t="str">
+      <c r="AK6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="49"/>
+      <c r="AL6" s="50"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="48" t="str">
+      <c r="AN6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="49"/>
+      <c r="AO6" s="50"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="48" t="str">
+      <c r="AQ6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="49"/>
+      <c r="AR6" s="50"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -15171,36 +14464,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15234,78 +14527,78 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="27" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="51" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="D4" s="47" t="s">
+      <c r="B4" s="51"/>
+      <c r="D4" s="51" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="47"/>
-      <c r="G4" s="47" t="s">
+      <c r="E4" s="51"/>
+      <c r="G4" s="51" t="s">
         <v>155</v>
       </c>
-      <c r="H4" s="47"/>
-      <c r="J4" s="47" t="s">
+      <c r="H4" s="51"/>
+      <c r="J4" s="51" t="s">
         <v>156</v>
       </c>
-      <c r="K4" s="47"/>
-      <c r="M4" s="47" t="s">
+      <c r="K4" s="51"/>
+      <c r="M4" s="51" t="s">
         <v>157</v>
       </c>
-      <c r="N4" s="47"/>
-      <c r="P4" s="47" t="s">
+      <c r="N4" s="51"/>
+      <c r="P4" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="Q4" s="47"/>
+      <c r="Q4" s="51"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="47" t="s">
+      <c r="S4" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="T4" s="47"/>
+      <c r="T4" s="51"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="47" t="s">
+      <c r="V4" s="51" t="s">
         <v>160</v>
       </c>
-      <c r="W4" s="47"/>
+      <c r="W4" s="51"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="47" t="s">
+      <c r="Y4" s="51" t="s">
         <v>161</v>
       </c>
-      <c r="Z4" s="47"/>
+      <c r="Z4" s="51"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="47" t="s">
+      <c r="AB4" s="51" t="s">
         <v>162</v>
       </c>
-      <c r="AC4" s="47"/>
-      <c r="AE4" s="47" t="s">
+      <c r="AC4" s="51"/>
+      <c r="AE4" s="51" t="s">
         <v>163</v>
       </c>
-      <c r="AF4" s="47"/>
+      <c r="AF4" s="51"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="47" t="s">
+      <c r="AH4" s="51" t="s">
         <v>164</v>
       </c>
-      <c r="AI4" s="47"/>
+      <c r="AI4" s="51"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="47" t="s">
+      <c r="AK4" s="51" t="s">
         <v>165</v>
       </c>
-      <c r="AL4" s="47"/>
+      <c r="AL4" s="51"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="47" t="s">
+      <c r="AN4" s="51" t="s">
         <v>166</v>
       </c>
-      <c r="AO4" s="47"/>
+      <c r="AO4" s="51"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="47" t="s">
+      <c r="AQ4" s="51" t="s">
         <v>167</v>
       </c>
-      <c r="AR4" s="47"/>
+      <c r="AR4" s="51"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="43" t="s">
@@ -16394,14 +15687,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -16418,12 +15709,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16789,19 +16082,24 @@
       <c r="N16" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E3:E42">
-    <cfRule type="expression" dxfId="2" priority="1">
-      <formula>OR($D3="Intercept", $D3="Radius")</formula>
+  <conditionalFormatting sqref="E4:E42">
+    <cfRule type="expression" dxfId="10" priority="4">
+      <formula>OR($D4="Intercept", $D4="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="0" priority="2">
+    <cfRule type="expression" dxfId="8" priority="2">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E3">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>

<commit_message>
update pile docs, samples, and SSRM upper bound handling
- Rewrite docs/fem/piles.md for full 6-DOF beam elements: mixed DOF
  system, moment extraction, plastic hinge, fixity, remove static
  condensation section
- Update docs/fem/samples.md pile problem: 1:1 slope, c=200/phi=20,
  two rows D=2 piles, V_cap=46000, M_cap=60000, FS 1.19->1.32
- Update docs/lem/samples.md pile problem: same geometry, FS 1.15->1.85,
  full Ito & Matsui summary with capacity checks, LEM vs FEM comparison
- Regenerate all sample figures for both LEM and FEM
- Improve LEM summary output: clearer capacity check reporting showing
  which limit controls and before/after capping
- Fix SSRM: return error when F_max still converges instead of
  reporting F_max as valid FS
- Read Fixity column from piles sheet in fileio.py

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fem/files/xslope_piles_fem.xlsx
+++ b/docs/fem/files/xslope_piles_fem.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/fem/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD98301-3702-904A-BF7A-4A97D6785FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75C80D43-D379-EA44-9AE9-C42B4915A2C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25040" yWindow="2500" windowWidth="42700" windowHeight="22800" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="29500" yWindow="9100" windowWidth="36220" windowHeight="22300" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="183">
   <si>
     <t>X</t>
   </si>
@@ -1252,56 +1252,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill>
@@ -1454,10 +1405,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>30</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>90</c:v>
+                  <c:v>80</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7895,10 +7846,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>10</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7910,7 +7861,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>6.67</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-10</c:v>
@@ -7970,6 +7921,12 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -7979,6 +7936,12 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-10</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -11311,13 +11274,13 @@
         <v>182</v>
       </c>
       <c r="C3" s="3">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D3" s="3">
-        <v>6.67</v>
+        <v>5</v>
       </c>
       <c r="E3" s="3">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F3" s="3">
         <v>-10</v>
@@ -11325,7 +11288,7 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" s="3">
         <v>6</v>
@@ -11336,10 +11299,10 @@
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" s="3">
-        <v>25000</v>
+        <v>46000</v>
       </c>
       <c r="O3" s="3">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="P3" s="3" t="s">
         <v>40</v>
@@ -11350,23 +11313,48 @@
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C4" s="3">
+        <v>10</v>
+      </c>
+      <c r="D4" s="3">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3">
+        <v>10</v>
+      </c>
+      <c r="F4" s="3">
+        <v>-10</v>
+      </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
+      <c r="I4" s="3">
+        <v>2</v>
+      </c>
+      <c r="J4" s="3">
+        <v>6</v>
+      </c>
+      <c r="K4" s="3">
+        <v>518400000</v>
+      </c>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
+      <c r="N4" s="3">
+        <v>46000</v>
+      </c>
+      <c r="O4" s="3">
+        <v>60000</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
@@ -12556,7 +12544,7 @@
         <v>200</v>
       </c>
       <c r="F9" s="3">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
@@ -12575,10 +12563,10 @@
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
       <c r="W9" s="3">
-        <v>500000</v>
+        <v>2000000</v>
       </c>
       <c r="X9" s="3">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
@@ -13255,63 +13243,33 @@
     <mergeCell ref="W7:X7"/>
     <mergeCell ref="R7:V7"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:F50">
-    <cfRule type="expression" dxfId="15" priority="9">
-      <formula>$D10="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G10:H50">
-    <cfRule type="expression" dxfId="14" priority="8">
-      <formula>$D10="mc"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I10:J50">
-    <cfRule type="expression" dxfId="13" priority="10">
-      <formula>$D10="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N10:N50">
-    <cfRule type="expression" dxfId="12" priority="12">
-      <formula>$D10="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O10:O50">
-    <cfRule type="expression" dxfId="11" priority="19">
-      <formula>$D10="mc"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P10:Q50">
-    <cfRule type="expression" dxfId="10" priority="14">
-      <formula>$D10="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F9">
-    <cfRule type="expression" dxfId="6" priority="1">
+  <conditionalFormatting sqref="F9:F50">
+    <cfRule type="expression" dxfId="8" priority="1">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9:H9">
-    <cfRule type="expression" dxfId="5" priority="2">
+  <conditionalFormatting sqref="G9:H50">
+    <cfRule type="expression" dxfId="7" priority="2">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I9:J9">
-    <cfRule type="expression" dxfId="4" priority="3">
+  <conditionalFormatting sqref="I9:J50">
+    <cfRule type="expression" dxfId="6" priority="3">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N9">
-    <cfRule type="expression" dxfId="3" priority="4">
+  <conditionalFormatting sqref="N9:N50">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O9">
-    <cfRule type="expression" dxfId="2" priority="6">
+  <conditionalFormatting sqref="O9:O50">
+    <cfRule type="expression" dxfId="4" priority="6">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P9:Q9">
-    <cfRule type="expression" dxfId="1" priority="5">
+  <conditionalFormatting sqref="P9:Q50">
+    <cfRule type="expression" dxfId="3" priority="5">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13809,7 +13767,7 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3">
         <v>20</v>
@@ -13853,7 +13811,7 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="B11" s="3">
         <v>20</v>
@@ -16155,24 +16113,19 @@
       <c r="N16" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E4:E42">
-    <cfRule type="expression" dxfId="9" priority="4">
-      <formula>OR($D4="Intercept", $D4="Radius")</formula>
+  <conditionalFormatting sqref="E3:E42">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="8" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="7" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E3">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>